<commit_message>
Se genera una rama para un solo sector economico y un solo producto, con el codigo adaptado a trabajar en el entorno local. Falta generar el modelo en el archivo .gcn para un solo sector y producto y adaptar el codigo en R para esa situación.
</commit_message>
<xml_diff>
--- a/macro_sam_2008_analisis.xlsx
+++ b/macro_sam_2008_analisis.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\francisco.henriquez\Mis documentos\proyectos\equilibrio_general\eq_general\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF307187-9196-4FAD-95DC-7A6E6674C675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11310"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="macro_sam_2008__simp_2" sheetId="11" r:id="rId1"/>
@@ -18,7 +19,20 @@
     <sheet name="macro_sam_2008_v1" sheetId="7" r:id="rId4"/>
     <sheet name="macro_sam_2008" sheetId="1" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -613,10 +627,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="170" formatCode="#,##0.0000000"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -1121,11 +1136,11 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="42" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1172,24 +1187,7 @@
     <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="26">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="22">
     <dxf>
       <fill>
         <patternFill>
@@ -1205,9 +1203,12 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
       <fill>
         <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1243,47 +1244,12 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1360,6 +1326,27 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1645,7 +1632,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
@@ -1737,7 +1724,7 @@
         <v>0</v>
       </c>
       <c r="N2" s="5">
-        <f>+SUM(B2:M2)</f>
+        <f t="shared" ref="N2:N13" si="0">+SUM(B2:M2)</f>
         <v>83.492336422509979</v>
       </c>
       <c r="O2" t="s">
@@ -1752,7 +1739,7 @@
       <c r="A3" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="11">
         <v>0</v>
       </c>
       <c r="C3" s="5">
@@ -1789,7 +1776,7 @@
         <v>24.362225892369995</v>
       </c>
       <c r="N3" s="5">
-        <f>+SUM(B3:M3)</f>
+        <f t="shared" si="0"/>
         <v>90.879313784761649</v>
       </c>
       <c r="P3" s="7"/>
@@ -1835,7 +1822,7 @@
         <v>0</v>
       </c>
       <c r="N4" s="5">
-        <f>+SUM(B4:M4)</f>
+        <f t="shared" si="0"/>
         <v>34.133031362509982</v>
       </c>
       <c r="Q4" s="7">
@@ -1884,7 +1871,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="5">
-        <f>+SUM(B5:M5)</f>
+        <f t="shared" si="0"/>
         <v>49.359305059999997</v>
       </c>
       <c r="Q5" s="7">
@@ -1921,7 +1908,8 @@
         <v>0</v>
       </c>
       <c r="J6" s="5">
-        <v>4.0619130575</v>
+        <f>4.0619130575+0.0272368961616536</f>
+        <v>4.0891499536616536</v>
       </c>
       <c r="K6" s="5">
         <v>0</v>
@@ -1933,8 +1921,8 @@
         <v>0</v>
       </c>
       <c r="N6" s="5">
-        <f>+SUM(B6:M6)</f>
-        <v>73.464109063600006</v>
+        <f t="shared" si="0"/>
+        <v>73.491345959761674</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.15">
@@ -1978,7 +1966,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="5">
-        <f>+SUM(B7:M7)</f>
+        <f t="shared" si="0"/>
         <v>36.953714519999998</v>
       </c>
     </row>
@@ -2023,7 +2011,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="5">
-        <f>+SUM(B8:M8)</f>
+        <f t="shared" si="0"/>
         <v>15.874814386000001</v>
       </c>
     </row>
@@ -2068,7 +2056,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="5">
-        <f>+SUM(B9:M9)</f>
+        <f t="shared" si="0"/>
         <v>7.4808834299999996</v>
       </c>
     </row>
@@ -2095,7 +2083,8 @@
         <v>1.5233916200000002</v>
       </c>
       <c r="H10" s="5">
-        <v>2.5385214375</v>
+        <f>2.5385214375+0.0272368961616536</f>
+        <v>2.5657583336616536</v>
       </c>
       <c r="I10" s="5">
         <v>0</v>
@@ -2113,8 +2102,8 @@
         <v>0</v>
       </c>
       <c r="N10" s="5">
-        <f>+SUM(B10:M10)</f>
-        <v>4.0619130575</v>
+        <f t="shared" si="0"/>
+        <v>4.0891499536616536</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.15">
@@ -2158,7 +2147,7 @@
         <v>0</v>
       </c>
       <c r="N11" s="5">
-        <f>+SUM(B11:M11)</f>
+        <f t="shared" si="0"/>
         <v>5.8828657</v>
       </c>
     </row>
@@ -2203,7 +2192,7 @@
         <v>0</v>
       </c>
       <c r="N12" s="5">
-        <f>+SUM(B12:M12)</f>
+        <f t="shared" si="0"/>
         <v>7.3869768858900002</v>
       </c>
       <c r="Q12" s="7">
@@ -2252,7 +2241,7 @@
         <v>0</v>
       </c>
       <c r="N13" s="5">
-        <f>+SUM(B13:M13)</f>
+        <f t="shared" si="0"/>
         <v>24.362225894000002</v>
       </c>
     </row>
@@ -2261,51 +2250,51 @@
         <v>21</v>
       </c>
       <c r="B14" s="5">
-        <f>+SUM(B2:B13)</f>
+        <f t="shared" ref="B14:M14" si="1">+SUM(B2:B13)</f>
         <v>83.492336422509979</v>
       </c>
       <c r="C14" s="5">
-        <f>+SUM(C2:C13)</f>
+        <f t="shared" si="1"/>
         <v>90.879313308399986</v>
       </c>
       <c r="D14" s="5">
-        <f>+SUM(D2:D13)</f>
+        <f t="shared" si="1"/>
         <v>34.133031370000005</v>
       </c>
       <c r="E14" s="5">
-        <f>+SUM(E2:E13)</f>
+        <f t="shared" si="1"/>
         <v>49.359305090000007</v>
       </c>
       <c r="F14" s="5">
-        <f>+SUM(F2:F13)</f>
+        <f t="shared" si="1"/>
         <v>73.491345959761659</v>
       </c>
       <c r="G14" s="5">
-        <f>+SUM(G2:G13)</f>
+        <f t="shared" si="1"/>
         <v>36.953714519999998</v>
       </c>
       <c r="H14" s="5">
-        <f>+SUM(H2:H13)</f>
-        <v>15.847577930230001</v>
+        <f t="shared" si="1"/>
+        <v>15.874814826391654</v>
       </c>
       <c r="I14" s="5">
-        <f>+SUM(I2:I13)</f>
+        <f t="shared" si="1"/>
         <v>7.4808834300000004</v>
       </c>
       <c r="J14" s="5">
-        <f>+SUM(J2:J13)</f>
-        <v>4.0619130575</v>
+        <f t="shared" si="1"/>
+        <v>4.0891499536616536</v>
       </c>
       <c r="K14" s="5">
-        <f>+SUM(K2:K13)</f>
+        <f t="shared" si="1"/>
         <v>5.8828657</v>
       </c>
       <c r="L14" s="5">
-        <f>+SUM(L2:L13)</f>
+        <f t="shared" si="1"/>
         <v>7.3869768860000002</v>
       </c>
       <c r="M14" s="5">
-        <f>+SUM(M2:M13)</f>
+        <f t="shared" si="1"/>
         <v>24.362225892369995</v>
       </c>
       <c r="N14" s="5">
@@ -2327,7 +2316,7 @@
         <v>49.359305059999997</v>
       </c>
       <c r="F16">
-        <v>73.464109063600006</v>
+        <v>73.491345959761674</v>
       </c>
       <c r="G16">
         <v>36.953714519999998</v>
@@ -2339,7 +2328,7 @@
         <v>7.4808834299999996</v>
       </c>
       <c r="J16">
-        <v>4.0619130575</v>
+        <v>4.0891499536616536</v>
       </c>
       <c r="K16">
         <v>5.8828657</v>
@@ -2349,6 +2338,56 @@
       </c>
       <c r="M16">
         <v>24.362225894000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.15">
+      <c r="B17" s="12">
+        <f>+B14-B16</f>
+        <v>0</v>
+      </c>
+      <c r="C17" s="12">
+        <f t="shared" ref="C17:M17" si="2">+C14-C16</f>
+        <v>-4.7636166300435434E-7</v>
+      </c>
+      <c r="D17" s="12">
+        <f t="shared" si="2"/>
+        <v>7.4900228241858713E-9</v>
+      </c>
+      <c r="E17" s="12">
+        <f t="shared" si="2"/>
+        <v>3.0000009587638488E-8</v>
+      </c>
+      <c r="F17" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G17" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H17" s="12">
+        <f t="shared" si="2"/>
+        <v>4.4039165381093426E-7</v>
+      </c>
+      <c r="I17" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J17" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K17" s="12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L17" s="12">
+        <f t="shared" si="2"/>
+        <v>1.1000000910144081E-10</v>
+      </c>
+      <c r="M17" s="12">
+        <f t="shared" si="2"/>
+        <v>-1.6300063521157426E-9</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.15">
@@ -2357,47 +2396,47 @@
         <v>0</v>
       </c>
       <c r="C18" s="2">
-        <f t="shared" ref="C18:M18" si="0">ROUND(C14-C16,1)</f>
+        <f t="shared" ref="C18:M18" si="3">ROUND(C14-C16,1)</f>
         <v>0</v>
       </c>
       <c r="D18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="E18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="F18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="I18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="J18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="L18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="M18" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -2426,7 +2465,7 @@
       <c r="F21" s="7"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.15">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="10" t="s">
         <v>194</v>
       </c>
       <c r="D22" s="7"/>
@@ -2434,7 +2473,7 @@
       <c r="F22" s="7"/>
       <c r="J22" s="7">
         <f>+J6-C39</f>
-        <v>4.0619130575</v>
+        <v>4.0891499536616536</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.15">
@@ -2442,12 +2481,15 @@
       <c r="H23" s="7"/>
       <c r="J23" s="7">
         <f>+H10-C39</f>
-        <v>2.5385214375</v>
+        <v>2.5657583336616536</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.15">
       <c r="B25">
         <v>1000000</v>
+      </c>
+      <c r="F25">
+        <v>2.723689616165359E-2</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.15">
@@ -2628,33 +2670,33 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:N14">
-    <cfRule type="cellIs" dxfId="25" priority="7" operator="notEqual">
+  <conditionalFormatting sqref="B20">
+    <cfRule type="cellIs" dxfId="21" priority="4" operator="notEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B43:B45">
+    <cfRule type="cellIs" dxfId="20" priority="3" operator="notEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B53:B55">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="notEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B60">
+    <cfRule type="cellIs" dxfId="18" priority="1" operator="notEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18:M18">
-    <cfRule type="cellIs" dxfId="24" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="6" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B20">
-    <cfRule type="cellIs" dxfId="23" priority="4" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B43:B45">
-    <cfRule type="cellIs" dxfId="22" priority="3" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B53:B55">
-    <cfRule type="cellIs" dxfId="21" priority="2" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B60">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="notEqual">
+  <conditionalFormatting sqref="B2:N14">
+    <cfRule type="cellIs" dxfId="16" priority="7" operator="notEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2664,7 +2706,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Y71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
@@ -2760,10 +2802,10 @@
       <c r="E2" s="5">
         <v>14.341871281889999</v>
       </c>
-      <c r="F2" s="12">
-        <v>0</v>
-      </c>
-      <c r="G2" s="12">
+      <c r="F2" s="11">
+        <v>0</v>
+      </c>
+      <c r="G2" s="11">
         <v>0</v>
       </c>
       <c r="H2" s="5">
@@ -2832,13 +2874,13 @@
       <c r="D3" s="5">
         <v>0</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>0</v>
       </c>
       <c r="F3" s="5">
         <v>19.770212353719991</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="11">
         <v>0</v>
       </c>
       <c r="H3" s="5">
@@ -2907,10 +2949,10 @@
       <c r="D4" s="5">
         <v>0</v>
       </c>
-      <c r="E4" s="12">
-        <v>0</v>
-      </c>
-      <c r="F4" s="12">
+      <c r="E4" s="11">
+        <v>0</v>
+      </c>
+      <c r="F4" s="11">
         <v>0</v>
       </c>
       <c r="G4" s="5">
@@ -2970,13 +3012,13 @@
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="12">
-        <v>0</v>
-      </c>
-      <c r="C5" s="12">
-        <v>0</v>
-      </c>
-      <c r="D5" s="12">
+      <c r="B5" s="11">
+        <v>0</v>
+      </c>
+      <c r="C5" s="11">
+        <v>0</v>
+      </c>
+      <c r="D5" s="11">
         <v>0</v>
       </c>
       <c r="E5" s="5">
@@ -3028,7 +3070,7 @@
       <c r="U5" s="5">
         <v>0.16482158305</v>
       </c>
-      <c r="V5" s="12"/>
+      <c r="V5" s="11"/>
       <c r="W5" s="5">
         <f t="shared" si="0"/>
         <v>14.60937084733</v>
@@ -3042,13 +3084,13 @@
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="12">
-        <v>0</v>
-      </c>
-      <c r="C6" s="12">
-        <v>0</v>
-      </c>
-      <c r="D6" s="12">
+      <c r="B6" s="11">
+        <v>0</v>
+      </c>
+      <c r="C6" s="11">
+        <v>0</v>
+      </c>
+      <c r="D6" s="11">
         <v>0</v>
       </c>
       <c r="E6" s="5">
@@ -3100,7 +3142,7 @@
       <c r="U6" s="5">
         <v>20.612622200999997</v>
       </c>
-      <c r="V6" s="12"/>
+      <c r="V6" s="11"/>
       <c r="W6" s="5">
         <f t="shared" si="0"/>
         <v>24.824325021429996</v>
@@ -3114,13 +3156,13 @@
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="12">
-        <v>0</v>
-      </c>
-      <c r="C7" s="12">
-        <v>0</v>
-      </c>
-      <c r="D7" s="12">
+      <c r="B7" s="11">
+        <v>0</v>
+      </c>
+      <c r="C7" s="11">
+        <v>0</v>
+      </c>
+      <c r="D7" s="11">
         <v>0</v>
       </c>
       <c r="E7" s="5">
@@ -3172,7 +3214,7 @@
       <c r="U7" s="5">
         <v>3.5847821083199998</v>
       </c>
-      <c r="V7" s="12"/>
+      <c r="V7" s="11"/>
       <c r="W7" s="5">
         <f t="shared" si="0"/>
         <v>51.445617916001666</v>
@@ -3514,12 +3556,12 @@
       <c r="O12" s="5">
         <v>5.8828657</v>
       </c>
-      <c r="P12" s="12"/>
-      <c r="Q12" s="12"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="11"/>
       <c r="R12" s="5">
         <v>7.3869768860000002</v>
       </c>
-      <c r="S12" s="12"/>
+      <c r="S12" s="11"/>
       <c r="T12" s="5">
         <v>0</v>
       </c>
@@ -3754,9 +3796,9 @@
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
       <c r="E16" s="5">
         <v>0</v>
       </c>
@@ -3823,7 +3865,7 @@
       <c r="B17" s="5">
         <v>0</v>
       </c>
-      <c r="C17" s="12"/>
+      <c r="C17" s="11"/>
       <c r="D17" s="5">
         <v>0</v>
       </c>
@@ -3974,9 +4016,9 @@
       <c r="D19" s="5">
         <v>0</v>
       </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
       <c r="H19" s="5">
         <v>0</v>
       </c>
@@ -4040,11 +4082,11 @@
       <c r="D20" s="5">
         <v>0</v>
       </c>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
       <c r="J20" s="5">
         <v>0</v>
       </c>
@@ -4147,7 +4189,7 @@
       <c r="S21" s="5">
         <v>0</v>
       </c>
-      <c r="T21" s="12"/>
+      <c r="T21" s="11"/>
       <c r="U21" s="5">
         <v>0</v>
       </c>
@@ -4220,7 +4262,7 @@
       <c r="T22" s="5">
         <v>0</v>
       </c>
-      <c r="U22" s="12"/>
+      <c r="U22" s="11"/>
       <c r="V22" s="5">
         <v>0</v>
       </c>
@@ -4492,7 +4534,7 @@
       <c r="J30" s="7"/>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.15">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="10" t="s">
         <v>178</v>
       </c>
       <c r="H31" s="7"/>
@@ -4794,38 +4836,33 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B23:W23 W2:W22">
-    <cfRule type="cellIs" dxfId="19" priority="7" operator="notEqual">
+  <conditionalFormatting sqref="B29:D29">
+    <cfRule type="cellIs" dxfId="15" priority="4" operator="notEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B52:D54">
+    <cfRule type="cellIs" dxfId="14" priority="3" operator="notEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B62:D64">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="notEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B69:D69">
+    <cfRule type="cellIs" dxfId="12" priority="1" operator="notEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:V27">
-    <cfRule type="cellIs" dxfId="18" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="6" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:V22">
-    <cfRule type="cellIs" dxfId="17" priority="5" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B29:D29">
-    <cfRule type="cellIs" dxfId="16" priority="4" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B52:D54">
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B62:D64">
-    <cfRule type="cellIs" dxfId="14" priority="2" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B69:D69">
-    <cfRule type="cellIs" dxfId="13" priority="1" operator="notEqual">
+  <conditionalFormatting sqref="B2:W23">
+    <cfRule type="cellIs" dxfId="10" priority="5" operator="notEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4835,7 +4872,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Y58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
@@ -5141,9 +5178,9 @@
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
       <c r="E5" s="5">
         <v>0</v>
       </c>
@@ -5193,7 +5230,7 @@
       <c r="U5" s="5">
         <v>0.16482158305</v>
       </c>
-      <c r="V5" s="12"/>
+      <c r="V5" s="11"/>
       <c r="W5" s="5">
         <f t="shared" si="0"/>
         <v>14.60937084733</v>
@@ -5207,9 +5244,9 @@
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
       <c r="E6" s="5">
         <v>0</v>
       </c>
@@ -5259,7 +5296,7 @@
       <c r="U6" s="5">
         <v>20.612622200999997</v>
       </c>
-      <c r="V6" s="12"/>
+      <c r="V6" s="11"/>
       <c r="W6" s="5">
         <f t="shared" si="0"/>
         <v>24.824325021429996</v>
@@ -5273,9 +5310,9 @@
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
       <c r="E7" s="5">
         <v>0</v>
       </c>
@@ -5325,7 +5362,7 @@
       <c r="U7" s="5">
         <v>3.5847821083199998</v>
       </c>
-      <c r="V7" s="12"/>
+      <c r="V7" s="11"/>
       <c r="W7" s="5">
         <f t="shared" si="0"/>
         <v>51.445617916001666</v>
@@ -5667,12 +5704,12 @@
       <c r="O12" s="5">
         <v>5.8828657</v>
       </c>
-      <c r="P12" s="12"/>
-      <c r="Q12" s="12"/>
+      <c r="P12" s="11"/>
+      <c r="Q12" s="11"/>
       <c r="R12" s="5">
         <v>7.3869768860000002</v>
       </c>
-      <c r="S12" s="12"/>
+      <c r="S12" s="11"/>
       <c r="T12" s="5">
         <v>0</v>
       </c>
@@ -5907,9 +5944,9 @@
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
       <c r="E16" s="5">
         <v>0</v>
       </c>
@@ -5976,7 +6013,7 @@
       <c r="B17" s="5">
         <v>0</v>
       </c>
-      <c r="C17" s="12"/>
+      <c r="C17" s="11"/>
       <c r="D17" s="5">
         <v>0</v>
       </c>
@@ -6127,9 +6164,9 @@
       <c r="D19" s="5">
         <v>0</v>
       </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
       <c r="H19" s="5">
         <v>0</v>
       </c>
@@ -6193,11 +6230,11 @@
       <c r="D20" s="5">
         <v>0</v>
       </c>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
       <c r="J20" s="5">
         <v>0</v>
       </c>
@@ -6300,7 +6337,7 @@
       <c r="S21" s="5">
         <v>0</v>
       </c>
-      <c r="T21" s="12"/>
+      <c r="T21" s="11"/>
       <c r="U21" s="5">
         <v>0</v>
       </c>
@@ -6373,7 +6410,7 @@
       <c r="T22" s="5">
         <v>0</v>
       </c>
-      <c r="U22" s="12"/>
+      <c r="U22" s="11"/>
       <c r="V22" s="5">
         <v>0</v>
       </c>
@@ -6645,7 +6682,7 @@
       <c r="J30" s="7"/>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.15">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="10" t="s">
         <v>178</v>
       </c>
       <c r="H31" s="7"/>
@@ -6836,21 +6873,6 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B23:W23 W2:W22">
-    <cfRule type="cellIs" dxfId="12" priority="5" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B27:V27">
-    <cfRule type="cellIs" dxfId="11" priority="4" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:V22">
-    <cfRule type="cellIs" dxfId="10" priority="3" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B29:D29">
     <cfRule type="cellIs" dxfId="9" priority="2" operator="notEqual">
       <formula>0</formula>
@@ -6861,13 +6883,23 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B27:V27">
+    <cfRule type="cellIs" dxfId="7" priority="4" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:W23">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="notEqual">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AA39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
@@ -8773,7 +8805,7 @@
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.15">
-      <c r="A31" s="11" t="s">
+      <c r="A31" s="10" t="s">
         <v>178</v>
       </c>
     </row>
@@ -8788,23 +8820,18 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B23:W23 W2:W22">
-    <cfRule type="cellIs" dxfId="7" priority="4" operator="notEqual">
+  <conditionalFormatting sqref="B29:D29">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="notEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:V27">
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:V22">
-    <cfRule type="cellIs" dxfId="5" priority="2" operator="notEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B29:D29">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="notEqual">
+  <conditionalFormatting sqref="B2:W23">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="notEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8814,7 +8841,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AA177"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
@@ -11533,7 +11560,7 @@
       <c r="E97" t="s">
         <v>154</v>
       </c>
-      <c r="H97" s="10"/>
+      <c r="H97" s="9"/>
     </row>
     <row r="98" spans="2:8" x14ac:dyDescent="0.15">
       <c r="B98" t="s">
@@ -11821,7 +11848,7 @@
       <c r="B133" t="s">
         <v>161</v>
       </c>
-      <c r="E133" s="9">
+      <c r="E133" s="8">
         <f>+E2</f>
         <v>28.80303928</v>
       </c>
@@ -11848,7 +11875,7 @@
       <c r="B136" t="s">
         <v>164</v>
       </c>
-      <c r="E136" s="8">
+      <c r="E136" s="7">
         <f>+E3</f>
         <v>0.17356569899999999</v>
       </c>
@@ -12218,23 +12245,18 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J50">
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="notEqual">
+  <conditionalFormatting sqref="B27:V27">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B23:W23 W2:W22">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="notEqual">
+  <conditionalFormatting sqref="B2:W23">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="notEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B27:V27">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:V22">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="notEqual">
+  <conditionalFormatting sqref="J50">
+    <cfRule type="cellIs" dxfId="0" priority="5" operator="notEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Se estimaron los parametros gamma y beta  aprtir de los datos y se mejoraron los resultados de partirda de la base de impuesto a la renta (PIT)
</commit_message>
<xml_diff>
--- a/macro_sam_2008_analisis.xlsx
+++ b/macro_sam_2008_analisis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\francisco.henriquez\Mis documentos\proyectos\equilibrio_general\eq_general\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF307187-9196-4FAD-95DC-7A6E6674C675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E9BA6AE-4475-47CE-BA8B-033AB67F8FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="macro_sam_2008__simp_2" sheetId="11" r:id="rId1"/>
@@ -19,6 +19,41 @@
     <sheet name="macro_sam_2008_v1" sheetId="7" r:id="rId4"/>
     <sheet name="macro_sam_2008" sheetId="1" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="solver_adj" localSheetId="0" hidden="1">macro_sam_2008__simp_2!$B$69</definedName>
+    <definedName name="solver_cvg" localSheetId="0" hidden="1">0.0001</definedName>
+    <definedName name="solver_drv" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_eng" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_est" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_itr" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_lhs1" localSheetId="0" hidden="1">macro_sam_2008__simp_2!$B$69</definedName>
+    <definedName name="solver_lhs2" localSheetId="0" hidden="1">macro_sam_2008__simp_2!$B$69</definedName>
+    <definedName name="solver_mip" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_mni" localSheetId="0" hidden="1">30</definedName>
+    <definedName name="solver_mrt" localSheetId="0" hidden="1">0.075</definedName>
+    <definedName name="solver_msl" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_neg" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_nod" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_opt" localSheetId="0" hidden="1">macro_sam_2008__simp_2!$F$67</definedName>
+    <definedName name="solver_pre" localSheetId="0" hidden="1">0.000001</definedName>
+    <definedName name="solver_rbv" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_rel2" localSheetId="0" hidden="1">3</definedName>
+    <definedName name="solver_rhs1" localSheetId="0" hidden="1">0.7</definedName>
+    <definedName name="solver_rhs2" localSheetId="0" hidden="1">0.3</definedName>
+    <definedName name="solver_rlx" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_rsd" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_scl" localSheetId="0" hidden="1">1</definedName>
+    <definedName name="solver_sho" localSheetId="0" hidden="1">2</definedName>
+    <definedName name="solver_ssz" localSheetId="0" hidden="1">100</definedName>
+    <definedName name="solver_tim" localSheetId="0" hidden="1">2147483647</definedName>
+    <definedName name="solver_tol" localSheetId="0" hidden="1">0.01</definedName>
+    <definedName name="solver_typ" localSheetId="0" hidden="1">3</definedName>
+    <definedName name="solver_val" localSheetId="0" hidden="1">0</definedName>
+    <definedName name="solver_ver" localSheetId="0" hidden="1">3</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="197">
   <si>
     <t>Act prim</t>
   </si>
@@ -622,6 +657,12 @@
   </si>
   <si>
     <t>Esta el la SAM que se está utilizando, con un solo producto producido en una sola actividad</t>
+  </si>
+  <si>
+    <t>beta</t>
+  </si>
+  <si>
+    <t>gamma</t>
   </si>
 </sst>
 </file>
@@ -631,7 +672,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="170" formatCode="#,##0.0000000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0000000"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -1140,7 +1181,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1633,7 +1674,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q62"/>
+  <dimension ref="A1:Q70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="4" width="12.5" bestFit="1" customWidth="1"/>
@@ -2667,6 +2708,64 @@
       <c r="B62" s="7">
         <f>+B60-B59</f>
         <v>1.1501183518899984</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A65" s="7" t="str">
+        <f>+A4</f>
+        <v>Trabajo</v>
+      </c>
+      <c r="B65" s="7">
+        <f>+B4</f>
+        <v>34.133031362509982</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A66" s="7" t="str">
+        <f>+A5</f>
+        <v>Capital</v>
+      </c>
+      <c r="B66" s="7">
+        <f>+B5</f>
+        <v>49.359305059999997</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A67" s="7" t="str">
+        <f>+A14</f>
+        <v>Total</v>
+      </c>
+      <c r="B67" s="7">
+        <f>+B14</f>
+        <v>83.492336422509979</v>
+      </c>
+      <c r="D67">
+        <f>B70*(65^B69)*(B66^(1-B69))</f>
+        <v>83.492336404101223</v>
+      </c>
+      <c r="F67" s="7">
+        <f>+B67-D67</f>
+        <v>1.8408755408927391E-8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A69" t="s">
+        <v>195</v>
+      </c>
+      <c r="B69">
+        <v>0.43654369057980391</v>
+      </c>
+      <c r="D69">
+        <f>1-B69</f>
+        <v>0.56345630942019609</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A70" t="s">
+        <v>196</v>
+      </c>
+      <c r="B70">
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se modifico el rol del IVA (se elimino de casi todas las ecuaciones en las que estaba ¿será correcto teoricamente?). Con eso mejora el ajutste, aunque aun no se llega a un equilibrio estable. El mayor error que queda es en las ecuaciones de condiciones de primer orden.
</commit_message>
<xml_diff>
--- a/macro_sam_2008_analisis.xlsx
+++ b/macro_sam_2008_analisis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\francisco.henriquez\Mis documentos\proyectos\equilibrio_general\eq_general\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E9BA6AE-4475-47CE-BA8B-033AB67F8FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A674702F-C876-41B9-8C9D-D2FD2EDF3154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="macro_sam_2008__simp_2" sheetId="11" r:id="rId1"/>
@@ -36,7 +36,7 @@
     <definedName name="solver_nod" localSheetId="0" hidden="1">2147483647</definedName>
     <definedName name="solver_num" localSheetId="0" hidden="1">2</definedName>
     <definedName name="solver_nwt" localSheetId="0" hidden="1">1</definedName>
-    <definedName name="solver_opt" localSheetId="0" hidden="1">macro_sam_2008__simp_2!$F$67</definedName>
+    <definedName name="solver_opt" localSheetId="0" hidden="1">macro_sam_2008__simp_2!$F$71</definedName>
     <definedName name="solver_pre" localSheetId="0" hidden="1">0.000001</definedName>
     <definedName name="solver_rbv" localSheetId="0" hidden="1">1</definedName>
     <definedName name="solver_rel1" localSheetId="0" hidden="1">1</definedName>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="198">
   <si>
     <t>Act prim</t>
   </si>
@@ -663,6 +663,9 @@
   </si>
   <si>
     <t>gamma</t>
+  </si>
+  <si>
+    <t>tasa vat</t>
   </si>
 </sst>
 </file>
@@ -1674,7 +1677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q70"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="10.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="4" width="12.5" bestFit="1" customWidth="1"/>
@@ -2710,7 +2713,7 @@
         <v>1.1501183518899984</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A65" s="7" t="str">
         <f>+A4</f>
         <v>Trabajo</v>
@@ -2720,7 +2723,7 @@
         <v>34.133031362509982</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A66" s="7" t="str">
         <f>+A5</f>
         <v>Capital</v>
@@ -2730,7 +2733,7 @@
         <v>49.359305059999997</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A67" s="7" t="str">
         <f>+A14</f>
         <v>Total</v>
@@ -2740,32 +2743,63 @@
         <v>83.492336422509979</v>
       </c>
       <c r="D67">
-        <f>B70*(65^B69)*(B66^(1-B69))</f>
-        <v>83.492336404101223</v>
+        <f>B70*(B65^B69)*(B66^(1-B69))</f>
+        <v>83.492336422509979</v>
       </c>
       <c r="F67" s="7">
         <f>+B67-D67</f>
-        <v>1.8408755408927391E-8</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.15">
+        <v>0</v>
+      </c>
+      <c r="H67">
+        <f>(B65^B69)*(B66^D69)</f>
+        <v>41.746166797763046</v>
+      </c>
+      <c r="J67">
+        <f>+B67/H67</f>
+        <v>2.0000000677184064</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A69" t="s">
         <v>195</v>
       </c>
       <c r="B69">
-        <v>0.43654369057980391</v>
+        <v>0.45415154287117893</v>
       </c>
       <c r="D69">
         <f>1-B69</f>
-        <v>0.56345630942019609</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.15">
+        <v>0.54584845712882113</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A70" t="s">
         <v>196</v>
       </c>
       <c r="B70">
-        <v>1.5</v>
+        <f>+J67</f>
+        <v>2.0000000677184064</v>
+      </c>
+      <c r="F70">
+        <f>+B70*B69*(B66^D69)*(B65^(B69-1))</f>
+        <v>1.1108938143082672</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="F71">
+        <f>+D69*B70*(B66^(D69-1))*(B65^B69)</f>
+        <v>0.92331451917543572</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.15">
+      <c r="A75" t="s">
+        <v>197</v>
+      </c>
+      <c r="B75">
+        <v>8.7999999999999995E-2</v>
+      </c>
+      <c r="D75">
+        <f>7.5+8.8+56</f>
+        <v>72.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>